<commit_message>
Added total votes column
</commit_message>
<xml_diff>
--- a/newjersey-election-2025/newjersey-election-results-2025.xlsx
+++ b/newjersey-election-2025/newjersey-election-results-2025.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/raddick/Documents/GitHub/election-cartograms/newjersey-election-2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E76896CF-9CFC-D74D-B913-583DD5D71E88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A3965CD-5CFE-BF43-B480-516909B5E8B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14060" yWindow="1060" windowWidth="27640" windowHeight="15600" xr2:uid="{4C8CBF91-8C8A-3149-A51A-57206E4F1A87}"/>
+    <workbookView xWindow="4080" yWindow="3360" windowWidth="27640" windowHeight="15600" xr2:uid="{4C8CBF91-8C8A-3149-A51A-57206E4F1A87}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="2" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="37">
   <si>
     <t>County</t>
   </si>
@@ -145,6 +145,9 @@
   </si>
   <si>
     <t>Ciattarelli</t>
+  </si>
+  <si>
+    <t>Total votes</t>
   </si>
 </sst>
 </file>
@@ -219,8 +222,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -556,24 +559,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A44A4D22-73B9-6D4E-A8C4-DF426876CAC2}">
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="9" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E1" s="9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="str">
         <f>Sheet1!A4</f>
         <v>Atlantic</v>
@@ -590,8 +596,12 @@
         <f>Sheet1!F4</f>
         <v>652</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E2" s="3">
+        <f>SUM(B2:D2)</f>
+        <v>99394</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="str">
         <f>Sheet1!A5</f>
         <v>Bergen</v>
@@ -608,8 +618,12 @@
         <f>Sheet1!F5</f>
         <v>1518</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E3" s="3">
+        <f t="shared" ref="E3:E22" si="0">SUM(B3:D3)</f>
+        <v>344661</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="str">
         <f>Sheet1!A6</f>
         <v>Burlington</v>
@@ -626,8 +640,12 @@
         <f>Sheet1!F6</f>
         <v>986</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E4" s="3">
+        <f t="shared" si="0"/>
+        <v>193106</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="str">
         <f>Sheet1!A7</f>
         <v>Camden</v>
@@ -644,8 +662,12 @@
         <f>Sheet1!F7</f>
         <v>1180</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E5" s="3">
+        <f t="shared" si="0"/>
+        <v>191980</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="str">
         <f>Sheet1!A8</f>
         <v>Cape May</v>
@@ -662,8 +684,12 @@
         <f>Sheet1!F8</f>
         <v>214</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E6" s="3">
+        <f t="shared" si="0"/>
+        <v>44069</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="str">
         <f>Sheet1!A9</f>
         <v>Cumberland</v>
@@ -680,8 +706,12 @@
         <f>Sheet1!F9</f>
         <v>290</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E7" s="3">
+        <f t="shared" si="0"/>
+        <v>40910</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="str">
         <f>Sheet1!A10</f>
         <v>Essex</v>
@@ -698,8 +728,12 @@
         <f>Sheet1!F10</f>
         <v>1118</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E8" s="3">
+        <f t="shared" si="0"/>
+        <v>245302</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="str">
         <f>Sheet1!A11</f>
         <v>Gloucester</v>
@@ -716,8 +750,12 @@
         <f>Sheet1!F11</f>
         <v>935</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E9" s="3">
+        <f t="shared" si="0"/>
+        <v>129266</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="str">
         <f>Sheet1!A12</f>
         <v>Hudson</v>
@@ -734,8 +772,12 @@
         <f>Sheet1!F12</f>
         <v>2122</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E10" s="3">
+        <f t="shared" si="0"/>
+        <v>170324</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="str">
         <f>Sheet1!A13</f>
         <v>Hunterdon</v>
@@ -752,8 +794,12 @@
         <f>Sheet1!F13</f>
         <v>401</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E11" s="3">
+        <f t="shared" si="0"/>
+        <v>66747</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="str">
         <f>Sheet1!A14</f>
         <v>Mercer</v>
@@ -770,8 +816,12 @@
         <f>Sheet1!F14</f>
         <v>741</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E12" s="3">
+        <f t="shared" si="0"/>
+        <v>128610</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="str">
         <f>Sheet1!A15</f>
         <v>Middlesex</v>
@@ -788,8 +838,12 @@
         <f>Sheet1!F15</f>
         <v>1992</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E13" s="3">
+        <f t="shared" si="0"/>
+        <v>277860</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="str">
         <f>Sheet1!A16</f>
         <v>Monmouth</v>
@@ -806,8 +860,12 @@
         <f>Sheet1!F16</f>
         <v>1503</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E14" s="3">
+        <f t="shared" si="0"/>
+        <v>287153</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="str">
         <f>Sheet1!A17</f>
         <v>Morris</v>
@@ -824,8 +882,12 @@
         <f>Sheet1!F17</f>
         <v>1006</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E15" s="3">
+        <f t="shared" si="0"/>
+        <v>228916</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="str">
         <f>Sheet1!A18</f>
         <v>Ocean</v>
@@ -842,8 +904,12 @@
         <f>Sheet1!F18</f>
         <v>1160</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E16" s="3">
+        <f t="shared" si="0"/>
+        <v>277440</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="str">
         <f>Sheet1!A19</f>
         <v>Passaic</v>
@@ -860,8 +926,12 @@
         <f>Sheet1!F19</f>
         <v>1081</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E17" s="3">
+        <f t="shared" si="0"/>
+        <v>149100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="str">
         <f>Sheet1!A20</f>
         <v>Salem</v>
@@ -878,8 +948,12 @@
         <f>Sheet1!F20</f>
         <v>192</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E18" s="3">
+        <f t="shared" si="0"/>
+        <v>23255</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="str">
         <f>Sheet1!A21</f>
         <v>Somerset</v>
@@ -896,8 +970,12 @@
         <f>Sheet1!F21</f>
         <v>1037</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E19" s="3">
+        <f t="shared" si="0"/>
+        <v>140487</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="str">
         <f>Sheet1!A22</f>
         <v>Sussex</v>
@@ -914,8 +992,12 @@
         <f>Sheet1!F22</f>
         <v>429</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E20" s="3">
+        <f t="shared" si="0"/>
+        <v>64851</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" t="str">
         <f>Sheet1!A23</f>
         <v>Union</v>
@@ -932,8 +1014,12 @@
         <f>Sheet1!F23</f>
         <v>1162</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E21" s="3">
+        <f t="shared" si="0"/>
+        <v>185278</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="str">
         <f>Sheet1!A24</f>
         <v>Warren</v>
@@ -949,6 +1035,10 @@
       <c r="D22">
         <f>Sheet1!F24</f>
         <v>326</v>
+      </c>
+      <c r="E22" s="3">
+        <f t="shared" si="0"/>
+        <v>45505</v>
       </c>
     </row>
   </sheetData>
@@ -962,7 +1052,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:10" ht="20" x14ac:dyDescent="0.2">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -974,15 +1064,15 @@
       <c r="D1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="20" x14ac:dyDescent="0.2">
-      <c r="A2" s="9"/>
+      <c r="A2" s="10"/>
       <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
@@ -992,8 +1082,8 @@
       <c r="D2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
     </row>
     <row r="3" spans="1:10" ht="20" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">

</xml_diff>

<commit_message>
Moved counties to look good
</commit_message>
<xml_diff>
--- a/newjersey-election-2025/newjersey-election-results-2025.xlsx
+++ b/newjersey-election-2025/newjersey-election-results-2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/raddick/Documents/GitHub/election-cartograms/newjersey-election-2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A3965CD-5CFE-BF43-B480-516909B5E8B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C53C225-8241-9E49-87CC-200F258B9DB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4080" yWindow="3360" windowWidth="27640" windowHeight="15600" xr2:uid="{4C8CBF91-8C8A-3149-A51A-57206E4F1A87}"/>
+    <workbookView xWindow="0" yWindow="1020" windowWidth="18900" windowHeight="15600" xr2:uid="{4C8CBF91-8C8A-3149-A51A-57206E4F1A87}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="2" r:id="rId1"/>
@@ -229,7 +229,28 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color theme="4"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1042,6 +1063,14 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A2:E22">
+    <cfRule type="expression" dxfId="1" priority="3">
+      <formula>$C2&gt;$B2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>$B2&gt;$C2</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>